<commit_message>
Mapping is almost ready
</commit_message>
<xml_diff>
--- a/docs/RAIS - Households.xlsx
+++ b/docs/RAIS - Households.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\amice13\GIT\idp-validator-ua\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D37B847-7DCE-478D-97FF-E06A9BA329EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A02507-BDBD-4BEE-9F99-F546B6FDEF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{7613FA96-0EF7-43B8-A86F-99DF97E351D5}"/>
   </bookViews>
@@ -111,6 +111,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -160,10 +163,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,7 +562,7 @@
       <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H2" t="s">

</xml_diff>